<commit_message>
Add automatic SSL/timeout fallbacks, First Run column, JS-shell detection, and crash fixes
</commit_message>
<xml_diff>
--- a/_MASTER_REPORTS/MASTER_SUMMARY.xlsx
+++ b/_MASTER_REPORTS/MASTER_SUMMARY.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:O63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,6 +484,11 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>First Run At</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>Last Run At</t>
         </is>
       </c>
@@ -491,17 +496,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NERC</t>
+          <t>AERC</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>335</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1230</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1168</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -513,55 +518,60 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>1230</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-08-29 18:43:09</t>
+          <t>2026-08-28T16:12:14</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-08-28 14:09:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PSERC</t>
+          <t>APERC</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1555</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1546</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -570,7 +580,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>1555</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -580,24 +590,29 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-08-29 18:43:14</t>
+          <t>2026-08-27T12:50:42</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-08-28 10:42:41</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RERC</t>
+          <t>APSERC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="D4" t="n">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -615,133 +630,148 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="L4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-08-31 11:10:42</t>
+          <t>2026-08-27T12:50:42</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-08-28 10:43:38</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TSERC</t>
+          <t>BERC</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>299</v>
+        <v>5000</v>
       </c>
       <c r="C5" t="n">
-        <v>5572</v>
+        <v>1823</v>
       </c>
       <c r="D5" t="n">
-        <v>5422</v>
+        <v>1807</v>
       </c>
       <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
         <v>2</v>
       </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" t="n">
-        <v>23</v>
-      </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>122</v>
+        <v>14</v>
       </c>
       <c r="K5" t="n">
-        <v>5522</v>
+        <v>1570</v>
       </c>
       <c r="L5" t="n">
-        <v>50</v>
+        <v>253</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-08-31 12:54:19</t>
+          <t>2026-08-27T12:50:42</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-08-28 14:15:40</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SSERC</t>
+          <t>CERC</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>105</v>
+        <v>21393</v>
       </c>
       <c r="D6" t="n">
-        <v>105</v>
+        <v>21068</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>151</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="K6" t="n">
-        <v>102</v>
+        <v>21160</v>
       </c>
       <c r="L6" t="n">
-        <v>3</v>
+        <v>125</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-08-31 10:23:28</t>
+          <t>2026-08-26T18:27:37</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-08-27 05:18:37</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>UERC</t>
+          <t>CP</t>
         </is>
       </c>
       <c r="B7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C7" t="n">
         <v>2</v>
       </c>
-      <c r="C7" t="n">
-        <v>8</v>
-      </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -762,7 +792,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -772,30 +802,35 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-08-29 11:18:33</t>
+          <t>2026-08-27T15:32:06</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-08-27 10:03:15</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TNERC</t>
+          <t>CSERC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>77</v>
+        <v>615</v>
       </c>
       <c r="C8" t="n">
-        <v>1088</v>
+        <v>1332</v>
       </c>
       <c r="D8" t="n">
-        <v>1087</v>
+        <v>1279</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -807,88 +842,98 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>1088</v>
+        <v>1332</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-08-31 13:13:49</t>
+          <t>2026-08-28T16:12:14</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-08-28 13:37:01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MERC</t>
+          <t>DERC</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>185</v>
+        <v>574</v>
       </c>
       <c r="C9" t="n">
-        <v>2063</v>
+        <v>3180</v>
       </c>
       <c r="D9" t="n">
-        <v>2032</v>
+        <v>2919</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>29</v>
+        <v>259</v>
       </c>
       <c r="K9" t="n">
-        <v>2041</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>22</v>
+        <v>3180</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-08-30 18:22:16</t>
+          <t>2026-08-28T16:47:29</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2026-08-29 09:03:34</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MERC-MSLDC</t>
+          <t>DOWN_TO_EARTH</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>186</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>2180</v>
+        <v>897</v>
       </c>
       <c r="D10" t="n">
-        <v>2131</v>
+        <v>870</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -897,43 +942,40 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="K10" t="n">
-        <v>2176</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2026-08-30 18:22:05</t>
-        </is>
-      </c>
+        <v>897</v>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MSERC</t>
+          <t>ERCKERALA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C11" t="n">
-        <v>427</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>397</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -951,43 +993,48 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>427</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-08-30 07:42:23</t>
+          <t>2026-08-28T16:47:29</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2026-08-28 11:18:08</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MPERC</t>
+          <t>GERC</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>254</v>
+        <v>5000</v>
       </c>
       <c r="C12" t="n">
-        <v>3191</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>3187</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -999,31 +1046,36 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>3149</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-08-30 18:24:20</t>
+          <t>2026-08-28T16:47:29</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2026-08-28 14:19:05</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>UPERC</t>
+          <t>HERC</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
@@ -1060,30 +1112,35 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-08-31 09:37:08</t>
+          <t>2026-08-28T16:47:29</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>2026-08-28 11:21:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WBERC</t>
+          <t>HPERC</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="C14" t="n">
-        <v>1638</v>
+        <v>1324</v>
       </c>
       <c r="D14" t="n">
-        <v>1636</v>
+        <v>1313</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -1095,140 +1152,147 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>1634</v>
+        <v>1297</v>
       </c>
       <c r="L14" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="M14" t="n">
         <v>0</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-08-31 10:01:41</t>
+          <t>2026-08-28T16:47:29</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>2026-08-28 11:41:31</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CEA</t>
+          <t>IEXINDIA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="C15" t="n">
-        <v>4472</v>
+        <v>516</v>
       </c>
       <c r="D15" t="n">
-        <v>4324</v>
+        <v>492</v>
       </c>
       <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>13</v>
+      </c>
+      <c r="K15" t="n">
+        <v>495</v>
+      </c>
+      <c r="L15" t="n">
+        <v>5</v>
+      </c>
+      <c r="M15" t="n">
         <v>16</v>
       </c>
-      <c r="F15" t="n">
-        <v>14</v>
-      </c>
-      <c r="G15" t="n">
-        <v>31</v>
-      </c>
-      <c r="H15" t="n">
-        <v>30</v>
-      </c>
-      <c r="I15" t="n">
-        <v>2</v>
-      </c>
-      <c r="J15" t="n">
-        <v>55</v>
-      </c>
-      <c r="K15" t="n">
-        <v>4332</v>
-      </c>
-      <c r="L15" t="n">
-        <v>140</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-08-31 06:38:03</t>
+          <t>2026-08-26T15:30:31</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>2026-08-27 07:31:49</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAG</t>
+          <t>MSTCE</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>3076</v>
+        <v>27</v>
       </c>
       <c r="D16" t="n">
-        <v>2998</v>
+        <v>24</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="G16" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>2965</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>111</v>
+        <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>2026-08-31 08:37:00</t>
-        </is>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>APTEL</t>
+          <t>ORIERC</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>44148</v>
+        <v>456</v>
       </c>
       <c r="D17" t="n">
-        <v>43827</v>
+        <v>378</v>
       </c>
       <c r="E17" t="n">
+        <v>16</v>
+      </c>
+      <c r="F17" t="n">
         <v>1</v>
       </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
@@ -1239,91 +1303,93 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>320</v>
+        <v>61</v>
       </c>
       <c r="K17" t="n">
-        <v>35622</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>8526</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>2026-08-31 08:56:53</t>
-        </is>
-      </c>
+        <v>456</v>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TERC</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>62</v>
+        <v>4509</v>
       </c>
       <c r="C18" t="n">
-        <v>45</v>
+        <v>4820</v>
       </c>
       <c r="D18" t="n">
-        <v>45</v>
+        <v>4793</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>45</v>
+        <v>4565</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>255</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-08-31 10:29:07</t>
+          <t>2026-08-27T12:09:49</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>2026-08-27 14:30:01</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DATAGOV</t>
+          <t>POWERMIN</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>126</v>
+        <v>87</v>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>191</v>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>191</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1338,34 +1404,39 @@
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>7</v>
+        <v>186</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M19" t="n">
         <v>0</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-08-31 12:55:16</t>
+          <t>2026-08-27T16:30:46</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2026-08-28 04:44:55</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FORUM_OF_REGULATORS</t>
+          <t>PRAPTI</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>103</v>
+        <v>16</v>
       </c>
       <c r="C20" t="n">
-        <v>542</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>524</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -1383,37 +1454,42 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>541</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
         <v>0</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-08-31 13:08:47</t>
+          <t>2026-08-28T17:11:50</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>2026-08-28 11:42:17</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GOV</t>
+          <t>SRPC</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -1425,13 +1501,13 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1440,28 +1516,25 @@
         <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>2026-09-01 08:01:45</t>
-        </is>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>JSERC</t>
+          <t>NERC</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>194</v>
+        <v>0</v>
       </c>
       <c r="C22" t="n">
-        <v>2961</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>2811</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -1470,7 +1543,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1479,34 +1552,39 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>2607</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>354</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
         <v>0</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-01 08:02:45</t>
+          <t>2026-08-29T16:43:29</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>2026-08-29 18:43:09</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NITI_FOR_STATES</t>
+          <t>PSERC</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -1527,193 +1605,213 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
         <v>0</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-01 08:30:37</t>
+          <t>2026-08-29T16:43:29</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-08-29 18:43:14</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NITI</t>
+          <t>RERC</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>511</v>
+        <v>58</v>
       </c>
       <c r="C24" t="n">
-        <v>1741</v>
+        <v>23</v>
       </c>
       <c r="D24" t="n">
-        <v>1725</v>
+        <v>20</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K24" t="n">
-        <v>1600</v>
+        <v>21</v>
       </c>
       <c r="L24" t="n">
-        <v>141</v>
+        <v>2</v>
       </c>
       <c r="M24" t="n">
         <v>0</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-01 09:19:54</t>
+          <t>2026-08-29T16:43:29</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>2026-08-31 11:10:42</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KPTCLSLDC</t>
+          <t>TSERC</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>27</v>
+        <v>299</v>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>5572</v>
       </c>
       <c r="D25" t="n">
-        <v>3</v>
+        <v>5422</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>5522</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-01 09:53:44</t>
+          <t>2026-08-29T16:46:55</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>2026-08-31 12:54:19</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>KERC</t>
+          <t>SSERC</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>664</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>8386</v>
+        <v>105</v>
       </c>
       <c r="D26" t="n">
-        <v>5269</v>
+        <v>105</v>
       </c>
       <c r="E26" t="n">
-        <v>324</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>401</v>
+        <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>230</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>2066</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>7961</v>
+        <v>102</v>
       </c>
       <c r="L26" t="n">
-        <v>425</v>
+        <v>3</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-01 12:05:54</t>
+          <t>2026-08-29T16:46:55</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2026-08-31 10:23:28</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PUNJABSLDC</t>
+          <t>UERC</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>70</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>9946</v>
+        <v>8</v>
       </c>
       <c r="D27" t="n">
-        <v>9650</v>
+        <v>8</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>291</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1722,40 +1820,45 @@
         <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>9932</v>
+        <v>8</v>
       </c>
       <c r="L27" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-01 12:11:20</t>
+          <t>2026-08-29T16:46:55</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>2026-08-29 11:18:33</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SLDC_MIZORAM</t>
+          <t>TNERC</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="C28" t="n">
-        <v>34</v>
+        <v>1088</v>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>1087</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1770,34 +1873,39 @@
         <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>7</v>
+        <v>1088</v>
       </c>
       <c r="M28" t="n">
         <v>0</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-01 12:33:43</t>
+          <t>2026-08-30T00:12:13</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2026-08-31 13:13:49</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SLDC_CG</t>
+          <t>MERC</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>95</v>
+        <v>185</v>
       </c>
       <c r="C29" t="n">
-        <v>162</v>
+        <v>2063</v>
       </c>
       <c r="D29" t="n">
-        <v>157</v>
+        <v>2032</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
@@ -1809,43 +1917,48 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="K29" t="n">
-        <v>161</v>
+        <v>2041</v>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="M29" t="n">
         <v>0</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-01 12:51:54</t>
+          <t>2026-08-30T12:20:30</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>2026-08-30 18:22:16</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SLDC_GUJ</t>
+          <t>MERC-MSLDC</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>227</v>
+        <v>186</v>
       </c>
       <c r="C30" t="n">
-        <v>665</v>
+        <v>2180</v>
       </c>
       <c r="D30" t="n">
-        <v>663</v>
+        <v>2131</v>
       </c>
       <c r="E30" t="n">
         <v>1</v>
@@ -1857,139 +1970,154 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="K30" t="n">
-        <v>580</v>
+        <v>2176</v>
       </c>
       <c r="L30" t="n">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="M30" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-01 13:28:41</t>
+          <t>2026-08-30T12:20:30</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>2026-08-30 18:22:05</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SLDC_ORISSA</t>
+          <t>MSERC</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>186</v>
+        <v>20</v>
       </c>
       <c r="C31" t="n">
-        <v>8478</v>
+        <v>427</v>
       </c>
       <c r="D31" t="n">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E31" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>5465</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>2573</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="K31" t="n">
-        <v>5876</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>2602</v>
+        <v>427</v>
       </c>
       <c r="M31" t="n">
         <v>0</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-01 14:21:13</t>
+          <t>2026-08-30T12:20:30</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>2026-08-30 07:42:23</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GRID-INDIA</t>
+          <t>MPERC</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>317</v>
+        <v>254</v>
       </c>
       <c r="C32" t="n">
-        <v>1219</v>
+        <v>3191</v>
       </c>
       <c r="D32" t="n">
-        <v>1159</v>
+        <v>3187</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" t="n">
+        <v>3149</v>
+      </c>
+      <c r="L32" t="n">
         <v>42</v>
       </c>
-      <c r="H32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" t="n">
-        <v>18</v>
-      </c>
-      <c r="K32" t="n">
-        <v>3</v>
-      </c>
-      <c r="L32" t="n">
-        <v>1216</v>
-      </c>
       <c r="M32" t="n">
         <v>0</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-01 15:35:32</t>
+          <t>2026-08-30T12:20:30</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>2026-08-30 18:24:20</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ASSAMSLDC</t>
+          <t>UPERC</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2887</v>
+        <v>1</v>
       </c>
       <c r="C33" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
@@ -1998,46 +2126,51 @@
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>94</v>
+        <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M33" t="n">
         <v>0</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-01 16:08:09</t>
+          <t>2026-08-31T00:05:57</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>2026-08-31 09:37:08</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>WBSLDC</t>
+          <t>WBERC</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>1914</v>
+        <v>1638</v>
       </c>
       <c r="D34" t="n">
-        <v>1087</v>
+        <v>1636</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
@@ -2046,145 +2179,160 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>805</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K34" t="n">
-        <v>1912</v>
+        <v>1634</v>
       </c>
       <c r="L34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M34" t="n">
         <v>0</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-02 06:54:39</t>
+          <t>2026-08-31T00:05:57</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>2026-08-31 10:01:41</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>WRLDC</t>
+          <t>CEA</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>268</v>
+        <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>143</v>
+        <v>4472</v>
       </c>
       <c r="D35" t="n">
+        <v>4324</v>
+      </c>
+      <c r="E35" t="n">
+        <v>16</v>
+      </c>
+      <c r="F35" t="n">
+        <v>14</v>
+      </c>
+      <c r="G35" t="n">
+        <v>31</v>
+      </c>
+      <c r="H35" t="n">
+        <v>30</v>
+      </c>
+      <c r="I35" t="n">
+        <v>2</v>
+      </c>
+      <c r="J35" t="n">
+        <v>55</v>
+      </c>
+      <c r="K35" t="n">
+        <v>4332</v>
+      </c>
+      <c r="L35" t="n">
         <v>140</v>
       </c>
-      <c r="E35" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" t="n">
-        <v>2</v>
-      </c>
-      <c r="G35" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" t="n">
-        <v>1</v>
-      </c>
-      <c r="K35" t="n">
-        <v>137</v>
-      </c>
-      <c r="L35" t="n">
-        <v>6</v>
-      </c>
       <c r="M35" t="n">
         <v>0</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-02 09:19:42</t>
+          <t>2026-08-31T11:27:19</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>2026-08-31 06:38:03</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TNEBSLDC</t>
+          <t>CAG</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2280</v>
+        <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>16306</v>
+        <v>3076</v>
       </c>
       <c r="D36" t="n">
-        <v>15707</v>
+        <v>2998</v>
       </c>
       <c r="E36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="G36" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="H36" t="n">
-        <v>364</v>
+        <v>7</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>214</v>
+        <v>33</v>
       </c>
       <c r="K36" t="n">
-        <v>16282</v>
+        <v>2965</v>
       </c>
       <c r="L36" t="n">
-        <v>24</v>
+        <v>111</v>
       </c>
       <c r="M36" t="n">
         <v>0</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-02 10:20:11</t>
+          <t>2026-08-31T11:27:19</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>2026-08-31 08:37:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CRISIL</t>
+          <t>APTEL</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>228</v>
+        <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>888</v>
+        <v>44148</v>
       </c>
       <c r="D37" t="n">
-        <v>888</v>
+        <v>43827</v>
       </c>
       <c r="E37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
@@ -2199,37 +2347,42 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="K37" t="n">
-        <v>817</v>
+        <v>35622</v>
       </c>
       <c r="L37" t="n">
-        <v>71</v>
+        <v>8526</v>
       </c>
       <c r="M37" t="n">
         <v>0</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-02 12:39:39</t>
+          <t>2026-08-31T11:27:19</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>2026-08-31 08:56:53</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>NRLDC</t>
+          <t>TERC</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>152</v>
+        <v>62</v>
       </c>
       <c r="C38" t="n">
-        <v>233</v>
+        <v>45</v>
       </c>
       <c r="D38" t="n">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
@@ -2247,68 +2400,1350 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>227</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="L38" t="n">
-        <v>233</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
         <v>0</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-02 16:03:35</t>
+          <t>2026-08-31T15:38:26</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>2026-08-31 10:29:07</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>DATAGOV</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>126</v>
+      </c>
+      <c r="C39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D39" t="n">
+        <v>6</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>7</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2026-08-31T17:38:33</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>2026-08-31 12:55:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>FORUM_OF_REGULATORS</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>103</v>
+      </c>
+      <c r="C40" t="n">
+        <v>542</v>
+      </c>
+      <c r="D40" t="n">
+        <v>524</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="n">
+        <v>18</v>
+      </c>
+      <c r="K40" t="n">
+        <v>541</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2026-08-31T17:49:16</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>2026-08-31 13:08:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>GOV</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026-09-01T13:31:13</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>2026-09-01 08:01:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>JSERC</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>194</v>
+      </c>
+      <c r="C42" t="n">
+        <v>2961</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2811</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>6</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>144</v>
+      </c>
+      <c r="K42" t="n">
+        <v>2607</v>
+      </c>
+      <c r="L42" t="n">
+        <v>354</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:24:46</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>2026-09-01 08:02:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>NITI_FOR_STATES</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>49</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>1</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-09-01T13:56:20</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>2026-09-01 08:30:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>NITI</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>511</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1741</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1725</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>5</v>
+      </c>
+      <c r="G44" t="n">
+        <v>5</v>
+      </c>
+      <c r="H44" t="n">
+        <v>4</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1600</v>
+      </c>
+      <c r="L44" t="n">
+        <v>141</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-08-27T13:01:51</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>2026-09-01 09:19:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>KPTCLSLDC</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>27</v>
+      </c>
+      <c r="C45" t="n">
+        <v>3</v>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>3</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-09-01T15:20:19</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>2026-09-01 09:53:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>KERC</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>664</v>
+      </c>
+      <c r="C46" t="n">
+        <v>8386</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5269</v>
+      </c>
+      <c r="E46" t="n">
+        <v>324</v>
+      </c>
+      <c r="F46" t="n">
+        <v>96</v>
+      </c>
+      <c r="G46" t="n">
+        <v>401</v>
+      </c>
+      <c r="H46" t="n">
+        <v>230</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>2066</v>
+      </c>
+      <c r="K46" t="n">
+        <v>7961</v>
+      </c>
+      <c r="L46" t="n">
+        <v>425</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:26:26</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>2026-09-01 12:05:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PUNJABSLDC</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>70</v>
+      </c>
+      <c r="C47" t="n">
+        <v>9946</v>
+      </c>
+      <c r="D47" t="n">
+        <v>9650</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>3</v>
+      </c>
+      <c r="H47" t="n">
+        <v>291</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>9932</v>
+      </c>
+      <c r="L47" t="n">
+        <v>14</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-09-01T15:58:47</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>2026-09-01 12:11:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SLDC_MIZORAM</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>38</v>
+      </c>
+      <c r="C48" t="n">
+        <v>34</v>
+      </c>
+      <c r="D48" t="n">
+        <v>34</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>27</v>
+      </c>
+      <c r="L48" t="n">
+        <v>7</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2026-09-01T18:00:47</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>2026-09-01 12:33:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SLDC_CG</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>95</v>
+      </c>
+      <c r="C49" t="n">
+        <v>162</v>
+      </c>
+      <c r="D49" t="n">
+        <v>157</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="n">
+        <v>5</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="n">
+        <v>161</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-09-01T18:02:04</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>2026-09-01 12:51:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SLDC_GUJ</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>227</v>
+      </c>
+      <c r="C50" t="n">
+        <v>665</v>
+      </c>
+      <c r="D50" t="n">
+        <v>663</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="n">
+        <v>1</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" t="n">
+        <v>580</v>
+      </c>
+      <c r="L50" t="n">
+        <v>85</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-09-01T18:07:39</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>2026-09-01 13:28:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SLDC_ORISSA</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>186</v>
+      </c>
+      <c r="C51" t="n">
+        <v>8478</v>
+      </c>
+      <c r="D51" t="n">
+        <v>399</v>
+      </c>
+      <c r="E51" t="n">
+        <v>13</v>
+      </c>
+      <c r="F51" t="n">
+        <v>5</v>
+      </c>
+      <c r="G51" t="n">
+        <v>5465</v>
+      </c>
+      <c r="H51" t="n">
+        <v>2573</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>23</v>
+      </c>
+      <c r="K51" t="n">
+        <v>5876</v>
+      </c>
+      <c r="L51" t="n">
+        <v>2602</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>2026-09-01T18:24:20</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>2026-09-01 14:21:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>GRID-INDIA</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>335</v>
+      </c>
+      <c r="C52" t="n">
+        <v>2473</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2290</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>67</v>
+      </c>
+      <c r="H52" t="n">
+        <v>40</v>
+      </c>
+      <c r="I52" t="n">
+        <v>43</v>
+      </c>
+      <c r="J52" t="n">
+        <v>33</v>
+      </c>
+      <c r="K52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L52" t="n">
+        <v>2470</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-09-01T13:51:42</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>2026-09-09 20:55:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ASSAMSLDC</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2887</v>
+      </c>
+      <c r="C53" t="n">
+        <v>96</v>
+      </c>
+      <c r="D53" t="n">
+        <v>87</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>3</v>
+      </c>
+      <c r="H53" t="n">
+        <v>1</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="n">
+        <v>5</v>
+      </c>
+      <c r="K53" t="n">
+        <v>94</v>
+      </c>
+      <c r="L53" t="n">
+        <v>2</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>2026-09-01T15:07:11</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>2026-09-01 16:08:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>WBSLDC</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>82</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1914</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1087</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" t="n">
+        <v>22</v>
+      </c>
+      <c r="H54" t="n">
+        <v>805</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1912</v>
+      </c>
+      <c r="L54" t="n">
+        <v>2</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>2026-09-02T11:45:41</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>2026-09-02 06:54:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>WRLDC</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>268</v>
+      </c>
+      <c r="C55" t="n">
+        <v>143</v>
+      </c>
+      <c r="D55" t="n">
+        <v>140</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="n">
+        <v>2</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" t="n">
+        <v>137</v>
+      </c>
+      <c r="L55" t="n">
+        <v>6</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>2026-09-02T12:01:26</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>2026-09-02 09:19:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>TNEBSLDC</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2280</v>
+      </c>
+      <c r="C56" t="n">
+        <v>16306</v>
+      </c>
+      <c r="D56" t="n">
+        <v>15707</v>
+      </c>
+      <c r="E56" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" t="n">
+        <v>18</v>
+      </c>
+      <c r="H56" t="n">
+        <v>364</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" t="n">
+        <v>214</v>
+      </c>
+      <c r="K56" t="n">
+        <v>16282</v>
+      </c>
+      <c r="L56" t="n">
+        <v>24</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>2026-09-02T11:44:14</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>2026-09-02 10:20:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CRISIL</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>228</v>
+      </c>
+      <c r="C57" t="n">
+        <v>888</v>
+      </c>
+      <c r="D57" t="n">
+        <v>888</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" t="n">
+        <v>817</v>
+      </c>
+      <c r="L57" t="n">
+        <v>71</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>2026-09-02T15:23:57</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>2026-09-02 12:39:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>NRLDC</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>154</v>
+      </c>
+      <c r="C58" t="n">
+        <v>310</v>
+      </c>
+      <c r="D58" t="n">
+        <v>6</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>304</v>
+      </c>
+      <c r="K58" t="n">
+        <v>227</v>
+      </c>
+      <c r="L58" t="n">
+        <v>83</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>2026-09-02T12:27:54</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>2026-09-07 12:56:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>BUSINESS_STANDARD</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B59" t="n">
         <v>10000</v>
       </c>
-      <c r="C39" t="n">
+      <c r="C59" t="n">
         <v>2853</v>
       </c>
-      <c r="D39" t="n">
+      <c r="D59" t="n">
         <v>2852</v>
       </c>
-      <c r="E39" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="n">
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" t="n">
         <v>1</v>
       </c>
-      <c r="K39" t="n">
+      <c r="K59" t="n">
         <v>2842</v>
       </c>
-      <c r="L39" t="n">
+      <c r="L59" t="n">
         <v>11</v>
       </c>
-      <c r="M39" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" t="inlineStr">
+      <c r="M59" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>2026-09-02T16:59:45</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
         <is>
           <t>2026-09-03 07:32:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>POWERMINT</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C60" t="n">
+        <v>166</v>
+      </c>
+      <c r="D60" t="n">
+        <v>166</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" t="n">
+        <v>77</v>
+      </c>
+      <c r="L60" t="n">
+        <v>89</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>2026-09-03T19:25:20</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>2026-09-04 14:03:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>GRIDCO</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>273</v>
+      </c>
+      <c r="C61" t="n">
+        <v>505</v>
+      </c>
+      <c r="D61" t="n">
+        <v>481</v>
+      </c>
+      <c r="E61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G61" t="n">
+        <v>2</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" t="n">
+        <v>18</v>
+      </c>
+      <c r="K61" t="n">
+        <v>472</v>
+      </c>
+      <c r="L61" t="n">
+        <v>33</v>
+      </c>
+      <c r="M61" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>2026-09-04T19:02:24</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>2026-09-04 14:13:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>MERCOM</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C62" t="n">
+        <v>338</v>
+      </c>
+      <c r="D62" t="n">
+        <v>332</v>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
+        <v>4</v>
+      </c>
+      <c r="K62" t="n">
+        <v>103</v>
+      </c>
+      <c r="L62" t="n">
+        <v>235</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>2026-09-02T17:02:47</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>2026-09-04 21:15:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>VASUDHA</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2680</v>
+      </c>
+      <c r="C63" t="n">
+        <v>530</v>
+      </c>
+      <c r="D63" t="n">
+        <v>522</v>
+      </c>
+      <c r="E63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="n">
+        <v>6</v>
+      </c>
+      <c r="K63" t="n">
+        <v>506</v>
+      </c>
+      <c r="L63" t="n">
+        <v>24</v>
+      </c>
+      <c r="M63" t="n">
+        <v>0</v>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>2026-09-07T16:25:49</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>2026-09-07 12:51:19</t>
         </is>
       </c>
     </row>

</xml_diff>